<commit_message>
Add nonfunctional performance and security tests
</commit_message>
<xml_diff>
--- a/VIPSportCenter_ReadyAPI_TestCases_Corrected.xlsx
+++ b/VIPSportCenter_ReadyAPI_TestCases_Corrected.xlsx
@@ -8,6 +8,10 @@
     <sheet name="Changes" sheetId="4" r:id="rId4"/>
     <sheet name="Results" sheetId="5" r:id="rId5"/>
     <sheet name="Defects" sheetId="6" r:id="rId6"/>
+    <sheet name="NFR Overview" sheetId="7" r:id="rIdNFR7"/>
+    <sheet name="NFR Cases" sheetId="8" r:id="rIdNFR8"/>
+    <sheet name="NFR Results" sheetId="9" r:id="rIdNFR9"/>
+    <sheet name="NFR Defects" sheetId="10" r:id="rIdNFR10"/>
   </sheets>
 </workbook>
 </file>
@@ -368,6 +372,207 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="90" customWidth="1"/>
+    <col min="5" max="5" width="95" customWidth="1"/>
+    <col min="6" max="6" width="100" customWidth="1"/>
+    <col min="7" max="7" width="90" customWidth="1"/>
+    <col min="8" max="8" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Case</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Severity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Policy / expected</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual evidence</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recommendation</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status / qualification</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFR-BUG-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-07</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Session write must verify planning.coach_id.
+Reuse owner seed planning; create new QA session 201; foreign coach POST 403/404; seanceRealisee remains null.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"attemptedStatus":200,"foreignWritePersisted":true}
+BOLA: foreign coach write accepted or persisted; HTTP=200, persisted=true</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/app/Http/Controllers/Coach/PlanningController.php::marquerRealisee</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify session planning coach ownership BEFORE updateOrCreate; reject 403/404.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detected in isolated lab; application NOT changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFR-BUG-002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-10</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROPOSED: invalid credentials should have indistinguishable public status/message.
+Unknown email and wrong password on QA account both 401 with identical message; this is not a timing side-channel test.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"unknownStatus":401,"knownStatus":401,"unknownMessage":"Incorrect email or password.","knownMessage":"Incorrect password. 4 attempt(s) remaining."}
+PROPOSED policy: account enumeration via different error messages
++ actual - expected
++ 'Incorrect email or password.'
+- 'Incorrect password. 4 attempt(s) remaining.'
+             ^
+</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/app/Http/Controllers/Auth/AuthController.php::login</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use generic invalid-credential public message; assess timing behavior separately.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detected in isolated lab; application NOT changed. Proposed policy gap; confirm requirements with team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFR-BUG-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-11</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium (proposed)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROPOSED LAB policy: &lt;=20 failed login attempts/minute/source; 429 by request 25.
+At most 25 sequential attempts with nonexistent unique email; at least one 429 and positive Retry-After. No real user lockout.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"attempts":25,"throttled":false,"retryAfter":null}
+PROPOSED lab anti-abuse policy: no 429 in bounded 25-request login burst</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/routes/api.php (login has no throttle middleware)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agree rate-limit policy; add throttle with persistent cache store for deployment, Retry-After and review reset/register routes.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detected in isolated lab; application NOT changed. Proposed policy gap; confirm requirements with team.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4"/>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:S34"/>
@@ -8967,4 +9172,3043 @@
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="115" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mục</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nội dung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scope</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33 original functional cases + 17 new NFR cases = 50; NFR includes 6 performance + 11 targeted security cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requirements/thresholds proposed for LAB. Existing functional cases unchanged. Original sheets are preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Node HTTP</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"total":17,"pass":14,"fail":3,"blocked":0} | 2026-10-05T07:38:22.125Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groovy scripts</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"total":17,"pass":13,"fail":4,"blocked":0} | 2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ReadyAPI Desktop</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run. XML schema/standalone Groovy evidence is NOT GUI evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Environment</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "managed": true,
+  "database": "fresh isolated seeded SQLite",
+  "server": "PHP built-in single-worker development server",
+  "php": "8.2.12",
+  "node": "v24.12.0",
+  "os": "win32 10.0.26200",
+  "cpu": "AMD Ryzen 7 H 255 w/ Radeon 780M Graphics",
+  "logicalCpus": 16,
+  "memoryGB": 30.8,
+  "bcryptRounds": 4
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thresholds</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p95: baseline 500ms; small load/mixed/stats 1000ms; spike 1500ms; short soak 750ms. All max 2000ms, errors 0. Not production SLOs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measurement</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full body latency with monotonic clock. Nearest-rank percentile. Main sample only; login/warmup/cleanup excluded. Throughput includes pacing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFR variables</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descriptions uniqueEmail/qaId/newSessionId/UTCtoday/role credentials are dynamic native script variables, not literal JSON values. Refer script for HTTP wire body. Standard admin fixture text applies only to cases that create a client; other cases follow the setup stated first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Safety</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">localhost only; explicit nfrLabOnly=true; max5 workers, &lt;=100 requests per phase, timeout5s. Login burst &lt;=25, nonexistent QA email only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isolation</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Managed mode creates fresh SQLite, migrate/seed, single-worker PHP server, BCRYPT_ROUNDS=4. Retains QA DB for evidence; stops owned server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code / commands</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">testing/nfr/run-nfr.mjs --managed; --category performance/security; --case TC-NFR-...; reports JSON/HTML/JUnit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ReadyAPI project</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">testing/VIPSportCenter-readyapi-project.xml: 50 cases/10 suites; testing/nfr/VIPSportCenter-nfr-readyapi-project.xml: 17 NFR cases/2 suites. Both use Groovy Script steps, not native Performance/Security Test UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual / future</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TLS/HSTS staging HTTPS; CORS/CSRF/XSS browser testing; native load UI; approved SLO and larger datasets; CPU/memory; long soak. Not executed here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limitation 1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only localhost and nfrLabOnly=true are accepted. Maximum 5 workers, 100 requests per batch, 5s per request; no external stress/DoS scans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limitation 2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PHP built-in development server is normally single-worker. Client concurrency is not proof of concurrent application processing; SQLite and seed dataset are small.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limitation 3</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Client-observed latency includes full response body; excludes login/setup, warmup and cleanup. Report nearest-rank p50/p95/p99, max, throughput and error rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limitation 4</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance targets and enumeration/throttle policies are proposed LAB requirements, not contractual production SLAs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limitation 5</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is bounded performance testing and targeted API security regression, not a complete pentest, certification, production capacity benchmark or long endurance test. Object-write probe creates a new QA session on an existing seeded planning; QA sessions remain in the disposable lab DB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limitation 6</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP localhost cannot validate TLS/HSTS. CORS, CSRF browser behavior, frontend XSS rendering, large production datasets, native ReadyAPI Load/Security Test UI and CPU/memory metrics remain untested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP source</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://owasp.org/API-Security/editions/2023/en/0x11-t10/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SmartBear source</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://support.smartbear.com/readyapi/getting-started/performance-testing/customizing-a-performance-test-part-1/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B23"/>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:O18"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="85" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="100" customWidth="1"/>
+    <col min="7" max="7" width="80" customWidth="1"/>
+    <col min="8" max="8" width="100" customWidth="1"/>
+    <col min="9" max="9" width="65" customWidth="1"/>
+    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requirement / proposed policy</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP mapping</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Profile / fixtures</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Method / endpoints</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expected / thresholds</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assertions</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cleanup / scope</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Node HTTP</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groovy script</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ReadyAPI GUI</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Candidate defect</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="150" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baseline /me: latency distribution</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAB target proposed by test team; validate with lecturer/product owner.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"routes":[{"role":"client","path":"/me"}],"warmup":5,"count":30,"concurrency":1}</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /me (client)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 + correct payload; p95 &lt;= 500ms; max &lt;= 2000ms; errorRate = 0.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status + payload for every sample; p50/p95/p99/max/RPS/errors; recovery per phase; min samples.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": {
+    "percentileMethod": "nearest-rank",
+    "phases": [
+      {
+        "phase": "measured",
+        "concurrency": 1,
+        "requests": 30,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 117.39,
+        "p95Ms": 149.25,
+        "p99Ms": 151.57,
+        "maxMs": 151.57,
+        "elapsedMs": 3767,
+        "throughputRps": 7.96
+      }
+    ]
+  },
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="150" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small concurrent load: admin client list</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAB target proposed by test team; validate with lecturer/product owner.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"routes":[{"role":"admin","path":"/admin/clients"}],"warmup":5,"count":50,"concurrency":5}</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /admin/clients (admin)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 + correct payload; p95 &lt;= 1000ms; max &lt;= 2000ms; errorRate = 0.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status + payload for every sample; p50/p95/p99/max/RPS/errors; recovery per phase; min samples.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": {
+    "percentileMethod": "nearest-rank",
+    "phases": [
+      {
+        "phase": "measured",
+        "concurrency": 5,
+        "requests": 50,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 793.62,
+        "p95Ms": 805.94,
+        "p99Ms": 810.14,
+        "maxMs": 810.14,
+        "elapsedMs": 7943,
+        "throughputRps": 6.3
+      }
+    ]
+  },
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mixed roles, read-only workload</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAB target proposed by test team; validate with lecturer/product owner.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"routes":[{"role":"admin","path":"/admin/clients"},{"role":"coach","path":"/coach/clients"},{"role":"client","path":"/client/paiements"}],"warmup":5,"count":60,"concurrency":3}</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /admin/clients (admin)
+GET /coach/clients (coach)
+GET /client/paiements (client)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 + correct payload; p95 &lt;= 1000ms; max &lt;= 2000ms; errorRate = 0.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status + payload for every sample; p50/p95/p99/max/RPS/errors; recovery per phase; min samples.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": {
+    "percentileMethod": "nearest-rank",
+    "phases": [
+      {
+        "phase": "measured",
+        "concurrency": 3,
+        "requests": 60,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 464.81,
+        "p95Ms": 485.38,
+        "p99Ms": 490.2,
+        "maxMs": 490.2,
+        "elapsedMs": 9300,
+        "throughputRps": 6.45
+      }
+    ]
+  },
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payment stats aggregation at small load</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAB target proposed by test team; validate with lecturer/product owner.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"routes":[{"role":"admin","path":"/admin/paiements/stats"}],"warmup":5,"count":30,"concurrency":3}</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /admin/paiements/stats (admin)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 + correct payload; p95 &lt;= 1000ms; max &lt;= 2000ms; errorRate = 0.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status + payload for every sample; p50/p95/p99/max/RPS/errors; recovery per phase; min samples.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": {
+    "percentileMethod": "nearest-rank",
+    "phases": [
+      {
+        "phase": "measured",
+        "concurrency": 3,
+        "requests": 30,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 419.41,
+        "p95Ms": 429.91,
+        "p99Ms": 430.43,
+        "maxMs": 430.43,
+        "elapsedMs": 4203,
+        "throughputRps": 7.14
+      }
+    ]
+  },
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bounded spike and recovery</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAB target proposed by test team; validate with lecturer/product owner.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"routes":[{"role":"admin","path":"/admin/clients"}],"warmup":5,"count":80,"concurrency":5,"phases":[{"name":"baseline","count":20,"concurrency":1},{"name":"spike","count":40,"concurrency":5},{"name":"recovery","count":20,"concurrency":1}]}</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /admin/clients (admin)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 + correct payload; p95 &lt;= 1500ms; max &lt;= 2000ms; errorRate = 0. Recovery p95 &lt;= max(500ms, 3 * baseline p95).</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status + payload for every sample; p50/p95/p99/max/RPS/errors; recovery per phase; min samples.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": {
+    "percentileMethod": "nearest-rank",
+    "phases": [
+      {
+        "phase": "baseline",
+        "concurrency": 1,
+        "requests": 20,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 158.27,
+        "p95Ms": 169.71,
+        "p99Ms": 171.98,
+        "maxMs": 171.98,
+        "elapsedMs": 3215,
+        "throughputRps": 6.22
+      },
+      {
+        "phase": "spike",
+        "concurrency": 5,
+        "requests": 40,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 793.78,
+        "p95Ms": 804.72,
+        "p99Ms": 805.89,
+        "maxMs": 805.89,
+        "elapsedMs": 6366,
+        "throughputRps": 6.28
+      },
+      {
+        "phase": "recovery",
+        "concurrency": 1,
+        "requests": 20,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 157.48,
+        "p95Ms": 166.21,
+        "p99Ms": 168.13,
+        "maxMs": 168.13,
+        "elapsedMs": 3174,
+        "throughputRps": 6.3
+      }
+    ],
+    "recoveryLimitMs": 509.13
+  },
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Short soak: 20 seconds, bounded requests</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAB target proposed by test team; validate with lecturer/product owner.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"routes":[{"role":"client","path":"/me"}],"warmup":5,"count":80,"concurrency":1,"durationMs":20000,"paceMs":250,"minimumSamples":20}</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /me (client)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 200 + correct payload; p95 &lt;= 750ms; max &lt;= 2000ms; errorRate = 0.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status + payload for every sample; p50/p95/p99/max/RPS/errors; recovery per phase; min samples.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": {
+    "percentileMethod": "nearest-rank",
+    "phases": [
+      {
+        "phase": "measured",
+        "concurrency": 1,
+        "requests": 79,
+        "errors": 0,
+        "errorRate": 0,
+        "p50Ms": 142.55,
+        "p95Ms": 154.16,
+        "p99Ms": 158.95,
+        "maxMs": 158.95,
+        "elapsedMs": 20033,
+        "throughputRps": 3.94
+      }
+    ]
+  },
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-01</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabricated Bearer token must be rejected</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reject unauthenticated API access.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API2:2023</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No login required.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /me; Bearer 999999|not-a-real-token; no body.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /me = 401; no user/profile data.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-02</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altered token must be rejected</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Token secret integrity must be enforced.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API2:2023</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Login client seed, retain original token; modify last secret character.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /login {email:clientEmail,password:clientPassword}; GET /me with changed token; GET /me with original token.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One-character changed token -&gt; 401; original token still works.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-03</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revoked token cannot be replayed</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logout invalidates this session token.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API2:2023</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issue dedicated client token; do not reuse other case tokens.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /login {email:clientEmail,password:clientPassword}; POST /logout with new token; GET /me with same revoked token.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Login 200; logout 200; reused token /me 401.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="75" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-04</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Role matrix blocks privileged reads and writes</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Client/coach cannot act as admin.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API5:2023</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin creates UUID QA client assigned to Karim; login admin/coach/client independently.
+Admin fixture: GET coach /me -&gt; POST admin/clients {prenom:"NFR",nom:"QA",email:uniqueEmail,password:"Password123!",coach_id:ownerProfileId,montant_annuel:3600}. Tokens/IDs from this case only.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /admin/clients as client then coach; PUT /admin/clients/{qaId} as client with {statut:"suspendu"}; GET same client as admin; require statut="actif".</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Client and coach admin reads 403; client PUT 403; QA client state unchanged.</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="75" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-05</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Registration role injection cannot grant admin</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public registration always grants client role.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API3:2023</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UUID email; admin token for cleanup only; register cash avoids payment mutation.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /register {name:"NFR QA",email:uniqueEmail,password:"Password123!",password_confirmation:"Password123!",specialite:"Musculation",plan:"mensuel",payment_method:"cash",role:"admin",active:true}; GET /me with returned token; GET /admin/clients with same token.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Submitted role=admin ignored/rejected; if created: /me role=client and admin access 403.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="75" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-06</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coach cannot read another coach client assessment</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assessments accessible only to assigned coach.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API1:2023</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin creates UUID QA client assigned to Sara (otherCoach); login Sara and Karim separately.
+Admin fixture: GET coach /me -&gt; POST admin/clients {prenom:"NFR",nom:"QA",email:uniqueEmail,password:"Password123!",coach_id:ownerProfileId,montant_annuel:3600}. Tokens/IDs from this case only.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /coach/clients/{qaId}/bilans as Sara (owner control200), then same URL as Karim (403/404).</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner read 200; other coach read 403 or 404; no assessment data.</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-07</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coach cannot mark another coach session completed</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Session write must verify planning.coach_id.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API1:2023</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Login Sara/Karim; read current-month planning as Sara; reuse an existing seeded planning/client. Create new QA session, never a seed session.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /coach/planning?mois={UTCmonth}&amp;annee={UTCyear} as Sara; POST /coach/planning/seances as Sara {client_id:ownerPlanning.client_id,date:UTCtoday,heure_debut:"10:00",heure_fin:"11:00",lieu:"NFR QA",notes:uniqueEmail}; GET planning before; POST /coach/seances/{newSessionId}/realiser as Karim {present:true,effort_percu:5,remarques_coach:"NFR unauthorized probe"}; GET planning as Sara after; compare seance_realisee.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reuse owner seed planning; create new QA session 201; foreign coach POST 403/404; seanceRealisee remains null.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFR-BUG-001</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {
+    "attemptedStatus": 200,
+    "foreignWritePersisted": true
+  },
+  "error": "BOLA: foreign coach write accepted or persisted; HTTP=200, persisted=true"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="75" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-08</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No password/hash/remember_token disclosure in JSON</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Responses must exclude authentication secrets at any nesting level.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API3:2023</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin creates UUID QA client; retain admin token for all three reads.
+Admin fixture: GET coach /me -&gt; POST admin/clients {prenom:"NFR",nom:"QA",email:uniqueEmail,password:"Password123!",coach_id:ownerProfileId,montant_annuel:3600}. Tokens/IDs from this case only.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GET /me; GET /admin/clients; GET /admin/clients/{qaId}; recursively inspect JSON field names, no raw response persisted.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recursive key check on /me, admin list and QA detail; no password, password_hash, remember_token, access_token or token.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="75" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-09</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Errors do not expose SQL, stack or source paths</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debug details must be suppressed (APP_DEBUG=false).</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API8:2023</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">APP_DEBUG=false, admin token only for protected missing-client URL.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /login {}; GET /admin/clients/2147483647 as admin; GET /nfr-route-not-found without token. Expected422/404/404.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invalid login 422, missing client 404 and unknown API 404; JSON with no trace/exception/file/SQLSTATE.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {},
+  "error": null
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-10</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Login does not reveal email existence</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROPOSED: invalid credentials should have indistinguishable public status/message.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API2:2023</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Admin creates UUID QA client; wrong-password only once, never seed account.
+Admin fixture: GET coach /me -&gt; POST admin/clients {prenom:"NFR",nom:"QA",email:uniqueEmail,password:"Password123!",coach_id:ownerProfileId,montant_annuel:3600}. Tokens/IDs from this case only.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POST /login {email:"absent-"+uniqueEmail,password:"Wrong123!"}; POST /login {email:uniqueEmail,password:"Wrong123!"}; compare public status/message.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown email and wrong password on QA account both 401 with identical message; this is not a timing side-channel test.</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFR-BUG-002</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {
+    "unknownStatus": 401,
+    "knownStatus": 401,
+    "unknownMessage": "Incorrect email or password.",
+    "knownMessage": "Incorrect password. 4 attempt(s) remaining."
+  },
+  "error": "PROPOSED policy: account enumeration via different error messages\n+ actual - expected\n\n+ 'Incorrect email or password.'\n- 'Incorrect password. 4 attempt(s) remaining.'\n             ^\n"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="135" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-11</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bounded login burst is throttled</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROPOSED LAB policy: &lt;=20 failed login attempts/minute/source; 429 by request 25.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OWASP API4:2023</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unique nonexistent QA email. No seeded-account login; max25 sequential requests, stop on first429.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repeat POST /login {email:uniqueEmail,password:"Wrong123!"}; expect429 by request25 and positive Retry-After.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At most 25 sequential attempts with nonexistent unique email; at least one 429 and positive Retry-After. No real user lockout.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact HTTP/access result + token/role/state/recursive JSON checks. See code action for all requests.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA client soft delete + logout issued tokens. Only lab DB; sessions/cotisations may remain.</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFR-BUG-003</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "metrics": null,
+  "observations": {
+    "attempts": 25,
+    "throttled": false,
+    "retryAfter": null
+  },
+  "error": "PROPOSED lab anti-abuse policy: no 429 in bounded 25-request login burst"
+}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O18"/>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K2:K18">
+      <formula1>"Not run,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L18">
+      <formula1>"Not run,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M2:M18">
+      <formula1>"Not run,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="90" customWidth="1"/>
+    <col min="6" max="6" width="100" customWidth="1"/>
+    <col min="7" max="7" width="65" customWidth="1"/>
+    <col min="8" max="8" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Node HTTP</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groovy script</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ReadyAPI GUI</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Node metrics / observations</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groovy metrics / observations</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run timestamps</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual error</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="150" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-01</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 1,
+      "requests": 30,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 117.39,
+      "p95Ms": 149.25,
+      "p99Ms": 151.57,
+      "maxMs": 151.57,
+      "elapsedMs": 3767,
+      "throughputRps": 7.96
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 1,
+      "requests": 30,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 121.66,
+      "p95Ms": 199.39,
+      "p99Ms": 222.24,
+      "maxMs": 222.24,
+      "elapsedMs": 4045,
+      "throughputRps": 7.42
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="150" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-02</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 5,
+      "requests": 50,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 793.62,
+      "p95Ms": 805.94,
+      "p99Ms": 810.14,
+      "maxMs": 810.14,
+      "elapsedMs": 7943,
+      "throughputRps": 6.3
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 5,
+      "requests": 50,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 949.04,
+      "p95Ms": 1049.27,
+      "p99Ms": 1071.79,
+      "maxMs": 1071.79,
+      "elapsedMs": 9624,
+      "throughputRps": 5.2
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p95 exceeds proposed lab target. Expression: (p.p95Ms &lt;= scenario.p95Ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-03</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 3,
+      "requests": 60,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 464.81,
+      "p95Ms": 485.38,
+      "p99Ms": 490.2,
+      "maxMs": 490.2,
+      "elapsedMs": 9300,
+      "throughputRps": 6.45
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 3,
+      "requests": 60,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 571,
+      "p95Ms": 616.68,
+      "p99Ms": 696.09,
+      "maxMs": 696.09,
+      "elapsedMs": 11439,
+      "throughputRps": 5.24
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 3,
+      "requests": 30,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 419.41,
+      "p95Ms": 429.91,
+      "p99Ms": 430.43,
+      "maxMs": 430.43,
+      "elapsedMs": 4203,
+      "throughputRps": 7.14
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 3,
+      "requests": 30,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 527.83,
+      "p95Ms": 602.84,
+      "p99Ms": 631.85,
+      "maxMs": 631.85,
+      "elapsedMs": 5363,
+      "throughputRps": 5.59
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-05</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "baseline",
+      "concurrency": 1,
+      "requests": 20,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 158.27,
+      "p95Ms": 169.71,
+      "p99Ms": 171.98,
+      "maxMs": 171.98,
+      "elapsedMs": 3215,
+      "throughputRps": 6.22
+    },
+    {
+      "phase": "spike",
+      "concurrency": 5,
+      "requests": 40,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 793.78,
+      "p95Ms": 804.72,
+      "p99Ms": 805.89,
+      "maxMs": 805.89,
+      "elapsedMs": 6366,
+      "throughputRps": 6.28
+    },
+    {
+      "phase": "recovery",
+      "concurrency": 1,
+      "requests": 20,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 157.48,
+      "p95Ms": 166.21,
+      "p99Ms": 168.13,
+      "maxMs": 168.13,
+      "elapsedMs": 3174,
+      "throughputRps": 6.3
+    }
+  ],
+  "recoveryLimitMs": 509.13
+}</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "baseline",
+      "concurrency": 1,
+      "requests": 20,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 177.79,
+      "p95Ms": 207.66,
+      "p99Ms": 248.21,
+      "maxMs": 248.21,
+      "elapsedMs": 3697,
+      "throughputRps": 5.41
+    },
+    {
+      "phase": "spike",
+      "concurrency": 5,
+      "requests": 40,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 956.74,
+      "p95Ms": 1011.43,
+      "p99Ms": 1022.67,
+      "maxMs": 1022.67,
+      "elapsedMs": 7697,
+      "throughputRps": 5.2
+    },
+    {
+      "phase": "recovery",
+      "concurrency": 1,
+      "requests": 20,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 191.65,
+      "p95Ms": 223.9,
+      "p99Ms": 226.32,
+      "maxMs": 226.32,
+      "elapsedMs": 3843,
+      "throughputRps": 5.2
+    }
+  ],
+  "recoveryLimitMs": 622.98
+}</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-PERF-06</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 1,
+      "requests": 79,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 142.55,
+      "p95Ms": 154.16,
+      "p99Ms": 158.95,
+      "maxMs": 158.95,
+      "elapsedMs": 20033,
+      "throughputRps": 3.94
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "percentileMethod": "nearest-rank",
+  "phases": [
+    {
+      "phase": "measured",
+      "concurrency": 1,
+      "requests": 79,
+      "errors": 0,
+      "errorRate": 0,
+      "p50Ms": 179.56,
+      "p95Ms": 206.99,
+      "p99Ms": 215.32,
+      "maxMs": 215.32,
+      "elapsedMs": 20136,
+      "throughputRps": 3.92
+    }
+  ]
+}</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-01</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-02</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-03</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-04</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-05</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-06</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-07</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "attemptedStatus": 200,
+  "foreignWritePersisted": true
+}</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "attemptedStatus": 200,
+  "foreignWritePersisted": true
+}</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BOLA: foreign coach write accepted or persisted; HTTP=200, persisted=true
+BOLA: foreign coach write accepted or persisted; HTTP=200, persisted=true. Expression: ((r.status in [403, 404]) &amp;&amp; observations.foreignWritePersisted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-08</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-09</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{}</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-10</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "unknownStatus": 401,
+  "knownStatus": 401,
+  "unknownMessage": "Incorrect email or password.",
+  "knownMessage": "Incorrect password. 4 attempt(s) remaining."
+}</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "unknownStatus": 401,
+  "knownStatus": 401,
+  "unknownMessage": "Incorrect email or password.",
+  "knownMessage": "Incorrect password. 4 attempt(s) remaining."
+}</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROPOSED policy: account enumeration via different error messages
++ actual - expected
++ 'Incorrect email or password.'
+- 'Incorrect password. 4 attempt(s) remaining.'
+             ^
+PROPOSED policy: account enumeration via different error messages. Expression: (unknown.data.message == known.data.message)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="75" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-NFR-SEC-11</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "attempts": 25,
+  "throttled": false,
+  "retryAfter": null
+}</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{
+  "attempts": 25,
+  "throttled": false,
+  "retryAfter": null
+}</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-05T07:38:22.125Z
+2026-10-05T07:44:17.498Z</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROPOSED lab anti-abuse policy: no 429 in bounded 25-request login burst
+PROPOSED lab anti-abuse policy: no 429 in bounded 25-request login burst. Expression: (limited != null). Values: limited = null</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H18"/>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B18">
+      <formula1>"Not run,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C18">
+      <formula1>"Not run,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D18">
+      <formula1>"Not run,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9"/>
+</worksheet>
 </file>
</xml_diff>